<commit_message>
Sync planning SharePoint : S28
</commit_message>
<xml_diff>
--- a/Plannings 2026 S28.xlsx
+++ b/Plannings 2026 S28.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{15FD9598-F048-44A4-8AB2-DEDBCAFB4389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{661953C8-8273-4104-8AFB-DE8C6C8416FC}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{15FD9598-F048-44A4-8AB2-DEDBCAFB4389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD23DD15-2834-43CD-98A8-C137E24A8955}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5801,7 +5801,7 @@
   <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="8" width="42.7109375" style="12" customWidth="1"/>
+    <col min="1" max="8" width="41.42578125" style="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7110,7 +7110,7 @@
     <mergeCell ref="B6:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="38" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="39" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -7877,13 +7877,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CB8547B6-5978-4AC9-9144-4303096A8128}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{678BE059-4D20-4ACB-A519-E73CE0A47114}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F43E0E8E-E1E4-4E8D-852C-AEA7BF6BF179}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F39E956-8F40-4CAF-87DD-7269CDEA3436}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E562B222-DF4D-4DE3-B7A1-2E025E2875CF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CDF86E59-6F43-4DEC-80A3-5A529498E295}"/>
 </file>
</xml_diff>